<commit_message>
test(automation): Playwright suites linked to the Excel test registers
New @workspace/qa-automation package covering all 119 cases from
docs/test-plans (109 automated, 9 manual-declared, 1 fixme):

- qcase() wrapper carries each Excel Case ID in the test title and a
  test-case annotation (the CR009 reporter's future upsert key), plus a
  per-suite tag (@smoke/@func/@neg/@e2e)
- global-setup bootstraps an idempotent world on the target instance:
  PW Automation project, PW-Alpha/PW-Beta modules, one actor per role
  (incl. a module-scoped qa_member for CR044 checks)
- suites: smoke (23, UI+API), functional (49), negative (35), e2e (12
  multi-actor journeys); Redmine/AI/mailbox cases self-skip or are
  declared manual so nothing is silently missing
- scripts/sync-traceability.py regenerates
  docs/test-plans/AUTOMATION_TRACEABILITY.md and writes the script link
  into each workbook's Additional/Comments column

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-plans/qapulse-e2e-tests.xlsx
+++ b/docs/test-plans/qapulse-e2e-tests.xlsx
@@ -1844,7 +1844,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -2190,7 +2190,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -2267,7 +2267,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -2300,7 +2300,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2404,7 +2404,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2458,7 +2458,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4080,7 +4080,11 @@
       </c>
       <c r="J2" s="177" t="inlineStr"/>
       <c r="K2" s="177" t="inlineStr"/>
-      <c r="L2" s="177" t="inlineStr"/>
+      <c r="L2" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:55</t>
+        </is>
+      </c>
       <c r="M2" s="177" t="inlineStr"/>
     </row>
     <row r="3">
@@ -4130,7 +4134,11 @@
       </c>
       <c r="J3" s="177" t="inlineStr"/>
       <c r="K3" s="177" t="inlineStr"/>
-      <c r="L3" s="177" t="inlineStr"/>
+      <c r="L3" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:155</t>
+        </is>
+      </c>
       <c r="M3" s="177" t="inlineStr"/>
     </row>
     <row r="4">
@@ -4181,7 +4189,11 @@
       </c>
       <c r="J4" s="177" t="inlineStr"/>
       <c r="K4" s="177" t="inlineStr"/>
-      <c r="L4" s="177" t="inlineStr"/>
+      <c r="L4" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:200</t>
+        </is>
+      </c>
       <c r="M4" s="177" t="inlineStr"/>
     </row>
     <row r="5">
@@ -4233,7 +4245,11 @@
       </c>
       <c r="J5" s="177" t="inlineStr"/>
       <c r="K5" s="177" t="inlineStr"/>
-      <c r="L5" s="177" t="inlineStr"/>
+      <c r="L5" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:237</t>
+        </is>
+      </c>
       <c r="M5" s="177" t="inlineStr"/>
     </row>
     <row r="6">
@@ -4285,7 +4301,11 @@
       </c>
       <c r="J6" s="177" t="inlineStr"/>
       <c r="K6" s="177" t="inlineStr"/>
-      <c r="L6" s="177" t="inlineStr"/>
+      <c r="L6" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:279</t>
+        </is>
+      </c>
       <c r="M6" s="177" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4335,7 +4355,11 @@
       </c>
       <c r="J7" s="177" t="inlineStr"/>
       <c r="K7" s="177" t="inlineStr"/>
-      <c r="L7" s="177" t="inlineStr"/>
+      <c r="L7" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:364</t>
+        </is>
+      </c>
       <c r="M7" s="177" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4385,7 +4409,11 @@
       </c>
       <c r="J8" s="177" t="inlineStr"/>
       <c r="K8" s="177" t="inlineStr"/>
-      <c r="L8" s="177" t="inlineStr"/>
+      <c r="L8" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:406</t>
+        </is>
+      </c>
       <c r="M8" s="177" t="inlineStr"/>
     </row>
     <row r="9">
@@ -4436,7 +4464,11 @@
       </c>
       <c r="J9" s="177" t="inlineStr"/>
       <c r="K9" s="177" t="inlineStr"/>
-      <c r="L9" s="177" t="inlineStr"/>
+      <c r="L9" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:463</t>
+        </is>
+      </c>
       <c r="M9" s="177" t="inlineStr"/>
     </row>
     <row r="10">
@@ -4487,7 +4519,11 @@
       </c>
       <c r="J10" s="177" t="inlineStr"/>
       <c r="K10" s="177" t="inlineStr"/>
-      <c r="L10" s="177" t="inlineStr"/>
+      <c r="L10" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:514</t>
+        </is>
+      </c>
       <c r="M10" s="177" t="inlineStr"/>
     </row>
     <row r="11">
@@ -4537,7 +4573,11 @@
       </c>
       <c r="J11" s="177" t="inlineStr"/>
       <c r="K11" s="177" t="inlineStr"/>
-      <c r="L11" s="177" t="inlineStr"/>
+      <c r="L11" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:566</t>
+        </is>
+      </c>
       <c r="M11" s="177" t="inlineStr"/>
     </row>
     <row r="12">
@@ -4587,7 +4627,11 @@
       </c>
       <c r="J12" s="177" t="inlineStr"/>
       <c r="K12" s="177" t="inlineStr"/>
-      <c r="L12" s="177" t="inlineStr"/>
+      <c r="L12" s="177" t="inlineStr">
+        <is>
+          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:604</t>
+        </is>
+      </c>
       <c r="M12" s="177" t="inlineStr"/>
     </row>
     <row r="13">
@@ -4637,7 +4681,11 @@
       </c>
       <c r="J13" s="177" t="inlineStr"/>
       <c r="K13" s="177" t="inlineStr"/>
-      <c r="L13" s="177" t="inlineStr"/>
+      <c r="L13" s="177" t="inlineStr">
+        <is>
+          <t>Manual (declared in spec as skip) — artifacts/qa-automation/tests/e2e.spec.ts:663</t>
+        </is>
+      </c>
       <c r="M13" s="177" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "test(automation): Playwright suites linked to the Excel test registers"
This reverts commit b25775c947326e3431d2da9efb10c2d9c0462f56.
</commit_message>
<xml_diff>
--- a/docs/test-plans/qapulse-e2e-tests.xlsx
+++ b/docs/test-plans/qapulse-e2e-tests.xlsx
@@ -1844,7 +1844,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -2190,7 +2190,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t>None</a:t>
+                <a:t/>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -2267,7 +2267,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t>None</a:t>
+                <a:t/>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -2300,7 +2300,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2404,7 +2404,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2458,7 +2458,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4080,11 +4080,7 @@
       </c>
       <c r="J2" s="177" t="inlineStr"/>
       <c r="K2" s="177" t="inlineStr"/>
-      <c r="L2" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:55</t>
-        </is>
-      </c>
+      <c r="L2" s="177" t="inlineStr"/>
       <c r="M2" s="177" t="inlineStr"/>
     </row>
     <row r="3">
@@ -4134,11 +4130,7 @@
       </c>
       <c r="J3" s="177" t="inlineStr"/>
       <c r="K3" s="177" t="inlineStr"/>
-      <c r="L3" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:155</t>
-        </is>
-      </c>
+      <c r="L3" s="177" t="inlineStr"/>
       <c r="M3" s="177" t="inlineStr"/>
     </row>
     <row r="4">
@@ -4189,11 +4181,7 @@
       </c>
       <c r="J4" s="177" t="inlineStr"/>
       <c r="K4" s="177" t="inlineStr"/>
-      <c r="L4" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:200</t>
-        </is>
-      </c>
+      <c r="L4" s="177" t="inlineStr"/>
       <c r="M4" s="177" t="inlineStr"/>
     </row>
     <row r="5">
@@ -4245,11 +4233,7 @@
       </c>
       <c r="J5" s="177" t="inlineStr"/>
       <c r="K5" s="177" t="inlineStr"/>
-      <c r="L5" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:237</t>
-        </is>
-      </c>
+      <c r="L5" s="177" t="inlineStr"/>
       <c r="M5" s="177" t="inlineStr"/>
     </row>
     <row r="6">
@@ -4301,11 +4285,7 @@
       </c>
       <c r="J6" s="177" t="inlineStr"/>
       <c r="K6" s="177" t="inlineStr"/>
-      <c r="L6" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:279</t>
-        </is>
-      </c>
+      <c r="L6" s="177" t="inlineStr"/>
       <c r="M6" s="177" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4355,11 +4335,7 @@
       </c>
       <c r="J7" s="177" t="inlineStr"/>
       <c r="K7" s="177" t="inlineStr"/>
-      <c r="L7" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:364</t>
-        </is>
-      </c>
+      <c r="L7" s="177" t="inlineStr"/>
       <c r="M7" s="177" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4409,11 +4385,7 @@
       </c>
       <c r="J8" s="177" t="inlineStr"/>
       <c r="K8" s="177" t="inlineStr"/>
-      <c r="L8" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:406</t>
-        </is>
-      </c>
+      <c r="L8" s="177" t="inlineStr"/>
       <c r="M8" s="177" t="inlineStr"/>
     </row>
     <row r="9">
@@ -4464,11 +4436,7 @@
       </c>
       <c r="J9" s="177" t="inlineStr"/>
       <c r="K9" s="177" t="inlineStr"/>
-      <c r="L9" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:463</t>
-        </is>
-      </c>
+      <c r="L9" s="177" t="inlineStr"/>
       <c r="M9" s="177" t="inlineStr"/>
     </row>
     <row r="10">
@@ -4519,11 +4487,7 @@
       </c>
       <c r="J10" s="177" t="inlineStr"/>
       <c r="K10" s="177" t="inlineStr"/>
-      <c r="L10" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:514</t>
-        </is>
-      </c>
+      <c r="L10" s="177" t="inlineStr"/>
       <c r="M10" s="177" t="inlineStr"/>
     </row>
     <row r="11">
@@ -4573,11 +4537,7 @@
       </c>
       <c r="J11" s="177" t="inlineStr"/>
       <c r="K11" s="177" t="inlineStr"/>
-      <c r="L11" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:566</t>
-        </is>
-      </c>
+      <c r="L11" s="177" t="inlineStr"/>
       <c r="M11" s="177" t="inlineStr"/>
     </row>
     <row r="12">
@@ -4627,11 +4587,7 @@
       </c>
       <c r="J12" s="177" t="inlineStr"/>
       <c r="K12" s="177" t="inlineStr"/>
-      <c r="L12" s="177" t="inlineStr">
-        <is>
-          <t>Automated — artifacts/qa-automation/tests/e2e.spec.ts:604</t>
-        </is>
-      </c>
+      <c r="L12" s="177" t="inlineStr"/>
       <c r="M12" s="177" t="inlineStr"/>
     </row>
     <row r="13">
@@ -4681,11 +4637,7 @@
       </c>
       <c r="J13" s="177" t="inlineStr"/>
       <c r="K13" s="177" t="inlineStr"/>
-      <c r="L13" s="177" t="inlineStr">
-        <is>
-          <t>Manual (declared in spec as skip) — artifacts/qa-automation/tests/e2e.spec.ts:663</t>
-        </is>
-      </c>
+      <c r="L13" s="177" t="inlineStr"/>
       <c r="M13" s="177" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: preserve local test-plan edits before upstream rename
These 4 files had skip-worktree set, silently hiding real local edits
from git for an unknown period. Committing under their current names
before merging in upstream's rename to qm-pulse-*.xlsx, so the local
content isn't discarded — content divergence needs a human call on
which version should carry over to the renamed files, not a guess.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-plans/qapulse-e2e-tests.xlsx
+++ b/docs/test-plans/qapulse-e2e-tests.xlsx
@@ -1844,7 +1844,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -2190,7 +2190,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -2267,7 +2267,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -2300,7 +2300,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2404,7 +2404,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2458,7 +2458,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4078,9 +4078,17 @@
           <t>Each stage transitions + notifies the right role; timeline shows Requirements-&gt;Develop-&gt;QA; verdict sent; milestone closed</t>
         </is>
       </c>
-      <c r="J2" s="177" t="inlineStr"/>
+      <c r="J2" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K2" s="177" t="inlineStr"/>
-      <c r="L2" s="177" t="inlineStr"/>
+      <c r="L2" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (3.1s) || Last automated run: 2026-07-19 03:30 UTC — Passed (2.9s)</t>
+        </is>
+      </c>
       <c r="M2" s="177" t="inlineStr"/>
     </row>
     <row r="3">
@@ -4128,9 +4136,17 @@
           <t>Author + PM notified on reject; re-review succeeds; final status approved; history shows the loop</t>
         </is>
       </c>
-      <c r="J3" s="177" t="inlineStr"/>
+      <c r="J3" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K3" s="177" t="inlineStr"/>
-      <c r="L3" s="177" t="inlineStr"/>
+      <c r="L3" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (1.1s) || Last automated run: 2026-07-19 03:30 UTC — Passed (1.2s)</t>
+        </is>
+      </c>
       <c r="M3" s="177" t="inlineStr"/>
     </row>
     <row r="4">
@@ -4179,9 +4195,17 @@
           <t>Dev + dev_lead notified on return; timeline resumes Develop same cycle then QA; final pass</t>
         </is>
       </c>
-      <c r="J4" s="177" t="inlineStr"/>
+      <c r="J4" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K4" s="177" t="inlineStr"/>
-      <c r="L4" s="177" t="inlineStr"/>
+      <c r="L4" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (1.3s) || Last automated run: 2026-07-19 03:30 UTC — Passed (1.6s)</t>
+        </is>
+      </c>
       <c r="M4" s="177" t="inlineStr"/>
     </row>
     <row r="5">
@@ -4231,9 +4255,17 @@
           <t>Status back to rejected-&gt;author; FA team notified; dev handoff reset; PM timeline shows a new Requirements cycle; completes</t>
         </is>
       </c>
-      <c r="J5" s="177" t="inlineStr"/>
+      <c r="J5" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K5" s="177" t="inlineStr"/>
-      <c r="L5" s="177" t="inlineStr"/>
+      <c r="L5" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (1.7s) || Last automated run: 2026-07-19 03:30 UTC — Passed (1.7s)</t>
+        </is>
+      </c>
       <c r="M5" s="177" t="inlineStr"/>
     </row>
     <row r="6">
@@ -4283,9 +4315,17 @@
           <t>Dev notified on assign; QA notified retest-needed; Dev notified on reopen (CR050); escape analysis reflects lifecycle</t>
         </is>
       </c>
-      <c r="J6" s="177" t="inlineStr"/>
+      <c r="J6" s="177" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
       <c r="K6" s="177" t="inlineStr"/>
-      <c r="L6" s="177" t="inlineStr"/>
+      <c r="L6" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Not Executed (0.3s) || Last automated run: 2026-07-19 03:30 UTC — Not Executed (0.3s)</t>
+        </is>
+      </c>
       <c r="M6" s="177" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4333,9 +4373,17 @@
           <t>Defect routed to author; author notified; handoff back works; requirement stays trackable</t>
         </is>
       </c>
-      <c r="J7" s="177" t="inlineStr"/>
+      <c r="J7" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K7" s="177" t="inlineStr"/>
-      <c r="L7" s="177" t="inlineStr"/>
+      <c r="L7" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (1.3s) || Last automated run: 2026-07-19 03:30 UTC — Passed (1.4s)</t>
+        </is>
+      </c>
       <c r="M7" s="177" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4383,9 +4431,17 @@
           <t>Member sees only A and B across all lists; C is not visible/accessible</t>
         </is>
       </c>
-      <c r="J8" s="177" t="inlineStr"/>
+      <c r="J8" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K8" s="177" t="inlineStr"/>
-      <c r="L8" s="177" t="inlineStr"/>
+      <c r="L8" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (2.7s) || Last automated run: 2026-07-19 03:30 UTC — Passed (3.0s)</t>
+        </is>
+      </c>
       <c r="M8" s="177" t="inlineStr"/>
     </row>
     <row r="9">
@@ -4434,9 +4490,17 @@
           <t>milestone_created-&gt;FA; submit-&gt;FA reviewers; approve-&gt;author+dev_lead; ready_for_qa-&gt;qa_lead - all module-scoped, HODs excluded</t>
         </is>
       </c>
-      <c r="J9" s="177" t="inlineStr"/>
+      <c r="J9" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K9" s="177" t="inlineStr"/>
-      <c r="L9" s="177" t="inlineStr"/>
+      <c r="L9" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (1.6s) || Last automated run: 2026-07-19 03:30 UTC — Passed (1.6s)</t>
+        </is>
+      </c>
       <c r="M9" s="177" t="inlineStr"/>
     </row>
     <row r="10">
@@ -4485,9 +4549,17 @@
           <t>Matrix shows Req -&gt; TCs -&gt; execution results with rolled-up coverage and pass state</t>
         </is>
       </c>
-      <c r="J10" s="177" t="inlineStr"/>
+      <c r="J10" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K10" s="177" t="inlineStr"/>
-      <c r="L10" s="177" t="inlineStr"/>
+      <c r="L10" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (0.7s) || Last automated run: 2026-07-19 03:30 UTC — Passed (0.6s)</t>
+        </is>
+      </c>
       <c r="M10" s="177" t="inlineStr"/>
     </row>
     <row r="11">
@@ -4535,9 +4607,17 @@
           <t>uat_milestone_ready notification fires to milestone PM at threshold; verdict sent</t>
         </is>
       </c>
-      <c r="J11" s="177" t="inlineStr"/>
+      <c r="J11" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K11" s="177" t="inlineStr"/>
-      <c r="L11" s="177" t="inlineStr"/>
+      <c r="L11" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (0.5s) || Last automated run: 2026-07-19 03:30 UTC — Passed (0.5s)</t>
+        </is>
+      </c>
       <c r="M11" s="177" t="inlineStr"/>
     </row>
     <row r="12">
@@ -4585,9 +4665,17 @@
           <t>Timeline shows repeating Requirements-&gt;Develop-&gt;QA cycles per bounce (not one flat window)</t>
         </is>
       </c>
-      <c r="J12" s="177" t="inlineStr"/>
+      <c r="J12" s="177" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="K12" s="177" t="inlineStr"/>
-      <c r="L12" s="177" t="inlineStr"/>
+      <c r="L12" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Passed (1.8s) || Last automated run: 2026-07-19 03:30 UTC — Passed (2.0s)</t>
+        </is>
+      </c>
       <c r="M12" s="177" t="inlineStr"/>
     </row>
     <row r="13">
@@ -4635,9 +4723,17 @@
           <t>Import maps fields; push creates issue (dedupe on retry CR051); status write-through + sync reconcile</t>
         </is>
       </c>
-      <c r="J13" s="177" t="inlineStr"/>
+      <c r="J13" s="177" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
       <c r="K13" s="177" t="inlineStr"/>
-      <c r="L13" s="177" t="inlineStr"/>
+      <c r="L13" s="177" t="inlineStr">
+        <is>
+          <t>Last automated run: 2026-07-19 03:02 UTC — Not Executed (0.0s) || Last automated run: 2026-07-19 03:30 UTC — Not Executed (0.0s)</t>
+        </is>
+      </c>
       <c r="M13" s="177" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>